<commit_message>
Close ELF at 76.17
Stop-loss triggered above the recorded 69.00 stop level (entry 74.00),
banking a small gain rather than a loss -- similar pattern to VERA's
trailing-stop exit. r_multiple +0.43R, pnl +EUR 2.49. followed_plan
and lesson still needed, flagged pink.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/data/TradingJournalCandidatesTry_updated.xlsx
+++ b/data/TradingJournalCandidatesTry_updated.xlsx
@@ -1576,9 +1576,23 @@
       <c r="Q13" s="7" t="n"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="T13" s="10" t="n">
+        <v>46205</v>
+      </c>
+      <c r="U13" t="n">
+        <v>76.17</v>
+      </c>
+      <c r="V13" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="X13" s="8" t="n"/>
+      <c r="Y13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>